<commit_message>
Calibrate beam cadence and affected enemy gates without changing growth
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/mon.xlsx
+++ b/space-battleship/config_excel/mon.xlsx
@@ -1056,22 +1056,22 @@
           <t>size</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>shieldType</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>shieldRecovery</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>shieldDelay</t>
         </is>
@@ -1118,22 +1118,22 @@
           <t>大小</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>独立护盾容量，随关卡生命倍率；0为无盾</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>护盾抗性类型：0无、1能量、2物理</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>每秒恢复最大盾量比例，受击暂停；0不恢复</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>有效命中后等待多少游戏秒才恢复</t>
         </is>
@@ -1180,22 +1180,22 @@
           <t>战场中占据的格子数</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1232,16 +1232,16 @@
       <c r="H4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
+      <c r="I4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1276,16 +1276,16 @@
       <c r="H5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
+      <c r="I5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1320,16 +1320,16 @@
       <c r="H6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
+      <c r="I6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1364,16 +1364,16 @@
       <c r="H7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="I7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1408,16 +1408,16 @@
       <c r="H8" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
+      <c r="I8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1452,16 +1452,16 @@
       <c r="H9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
+      <c r="I9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1496,16 +1496,16 @@
       <c r="H10" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
+      <c r="I10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1540,16 +1540,16 @@
       <c r="H11" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
+      <c r="I11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1584,16 +1584,16 @@
       <c r="H12" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
+      <c r="I12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1628,16 +1628,16 @@
       <c r="H13" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
+      <c r="I13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1672,16 +1672,16 @@
       <c r="H14" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
+      <c r="I14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1716,16 +1716,16 @@
       <c r="H15" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
+      <c r="I15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1760,16 +1760,16 @@
       <c r="H16" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
+      <c r="I16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1804,16 +1804,16 @@
       <c r="H17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
+      <c r="I17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1848,16 +1848,16 @@
       <c r="H18" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
+      <c r="I18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1892,16 +1892,16 @@
       <c r="H19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
+      <c r="I19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1936,16 +1936,16 @@
       <c r="H20" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
+      <c r="I20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1980,16 +1980,16 @@
       <c r="H21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
+      <c r="I21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2024,16 +2024,16 @@
       <c r="H22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
+      <c r="I22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2068,16 +2068,16 @@
       <c r="H23" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
+      <c r="I23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2112,16 +2112,16 @@
       <c r="H24" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
+      <c r="I24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2156,16 +2156,16 @@
       <c r="H25" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
+      <c r="I25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2200,16 +2200,16 @@
       <c r="H26" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
+      <c r="I26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2244,16 +2244,16 @@
       <c r="H27" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
+      <c r="I27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2288,16 +2288,16 @@
       <c r="H28" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="n">
+      <c r="I28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2332,16 +2332,16 @@
       <c r="H29" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="n">
+      <c r="I29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2376,16 +2376,16 @@
       <c r="H30" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
+      <c r="I30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2420,16 +2420,16 @@
       <c r="H31" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="n">
+      <c r="I31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2464,16 +2464,16 @@
       <c r="H32" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I32" t="n">
+      <c r="I32" s="1" t="n">
         <v>8000</v>
       </c>
-      <c r="J32" t="n">
-        <v>2</v>
-      </c>
-      <c r="K32" t="n">
+      <c r="J32" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" s="1" t="n">
         <v>0.2</v>
       </c>
-      <c r="L32" t="n">
+      <c r="L32" s="1" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -2508,16 +2508,16 @@
       <c r="H33" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I33" t="n">
+      <c r="I33" s="1" t="n">
         <v>8000</v>
       </c>
-      <c r="J33" t="n">
-        <v>2</v>
-      </c>
-      <c r="K33" t="n">
+      <c r="J33" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="1" t="n">
         <v>0.2</v>
       </c>
-      <c r="L33" t="n">
+      <c r="L33" s="1" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -2552,16 +2552,16 @@
       <c r="H34" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="n">
+      <c r="I34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2596,16 +2596,16 @@
       <c r="H35" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="n">
+      <c r="I35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2640,16 +2640,16 @@
       <c r="H36" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" t="n">
+      <c r="I36" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2684,16 +2684,16 @@
       <c r="H37" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" t="n">
+      <c r="I37" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2728,16 +2728,16 @@
       <c r="H38" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" t="n">
+      <c r="I38" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2772,16 +2772,16 @@
       <c r="H39" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="n">
-        <v>0</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" t="n">
+      <c r="I39" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2816,16 +2816,16 @@
       <c r="H40" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I40" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" t="n">
-        <v>0</v>
-      </c>
-      <c r="L40" t="n">
+      <c r="I40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2860,16 +2860,16 @@
       <c r="H41" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I41" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" t="n">
-        <v>0</v>
-      </c>
-      <c r="K41" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" t="n">
+      <c r="I41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2904,16 +2904,16 @@
       <c r="H42" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0</v>
-      </c>
-      <c r="L42" t="n">
+      <c r="I42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2948,16 +2948,16 @@
       <c r="H43" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0</v>
-      </c>
-      <c r="L43" t="n">
+      <c r="I43" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2992,16 +2992,16 @@
       <c r="H44" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I44" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" t="n">
+      <c r="I44" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3036,16 +3036,16 @@
       <c r="H45" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I45" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" t="n">
+      <c r="I45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3080,16 +3080,16 @@
       <c r="H46" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I46" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" t="n">
+      <c r="I46" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3124,16 +3124,16 @@
       <c r="H47" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" t="n">
+      <c r="I47" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3168,16 +3168,16 @@
       <c r="H48" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I48" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" t="n">
-        <v>0</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" t="n">
+      <c r="I48" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3212,16 +3212,16 @@
       <c r="H49" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I49" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" t="n">
-        <v>0</v>
-      </c>
-      <c r="K49" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" t="n">
+      <c r="I49" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3256,16 +3256,16 @@
       <c r="H50" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I50" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" t="n">
+      <c r="I50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3300,16 +3300,16 @@
       <c r="H51" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I51" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" t="n">
+      <c r="I51" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3344,16 +3344,16 @@
       <c r="H52" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I52" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" t="n">
-        <v>0</v>
-      </c>
-      <c r="K52" t="n">
-        <v>0</v>
-      </c>
-      <c r="L52" t="n">
+      <c r="I52" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3388,16 +3388,16 @@
       <c r="H53" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" t="n">
-        <v>0</v>
-      </c>
-      <c r="L53" t="n">
+      <c r="I53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3432,16 +3432,16 @@
       <c r="H54" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" t="n">
+      <c r="I54" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3476,16 +3476,16 @@
       <c r="H55" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I55" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" t="n">
+      <c r="I55" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3520,16 +3520,16 @@
       <c r="H56" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I56" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" t="n">
+      <c r="I56" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3564,16 +3564,16 @@
       <c r="H57" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" t="n">
+      <c r="I57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
         <v>7.5</v>
       </c>
       <c r="E58" s="1" t="n">
-        <v>32000</v>
+        <v>22800</v>
       </c>
       <c r="F58" s="1" t="n">
         <v>2</v>
@@ -3608,16 +3608,16 @@
       <c r="H58" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I58" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J58" t="n">
-        <v>2</v>
-      </c>
-      <c r="K58" t="n">
+      <c r="I58" s="1" t="n">
+        <v>22800</v>
+      </c>
+      <c r="J58" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" s="1" t="n">
         <v>0.2</v>
       </c>
-      <c r="L58" t="n">
+      <c r="L58" s="1" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
         <v>7.5</v>
       </c>
       <c r="E59" s="1" t="n">
-        <v>25000</v>
+        <v>17800</v>
       </c>
       <c r="F59" s="1" t="n">
         <v>2</v>
@@ -3652,16 +3652,16 @@
       <c r="H59" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I59" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J59" t="n">
-        <v>2</v>
-      </c>
-      <c r="K59" t="n">
+      <c r="I59" s="1" t="n">
+        <v>17800</v>
+      </c>
+      <c r="J59" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K59" s="1" t="n">
         <v>0.2</v>
       </c>
-      <c r="L59" t="n">
+      <c r="L59" s="1" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
         <v>0.1</v>
       </c>
       <c r="E60" s="1" t="n">
-        <v>17000</v>
+        <v>16000</v>
       </c>
       <c r="F60" s="1" t="n">
         <v>2</v>
@@ -3696,16 +3696,16 @@
       <c r="H60" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I60" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" t="n">
-        <v>0</v>
-      </c>
-      <c r="K60" t="n">
-        <v>0</v>
-      </c>
-      <c r="L60" t="n">
+      <c r="I60" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3724,10 +3724,10 @@
         </is>
       </c>
       <c r="D61" s="1" t="n">
-        <v>7.1</v>
+        <v>12</v>
       </c>
       <c r="E61" s="1" t="n">
-        <v>10000</v>
+        <v>21000</v>
       </c>
       <c r="F61" s="1" t="n">
         <v>2</v>
@@ -3740,16 +3740,16 @@
       <c r="H61" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I61" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" t="n">
-        <v>0</v>
-      </c>
-      <c r="L61" t="n">
+      <c r="I61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3768,10 +3768,10 @@
         </is>
       </c>
       <c r="D62" s="1" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="E62" s="1" t="n">
-        <v>7000</v>
+        <v>11100</v>
       </c>
       <c r="F62" s="1" t="n">
         <v>1</v>
@@ -3784,16 +3784,16 @@
       <c r="H62" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I62" t="n">
-        <v>0</v>
-      </c>
-      <c r="J62" t="n">
-        <v>0</v>
-      </c>
-      <c r="K62" t="n">
-        <v>0</v>
-      </c>
-      <c r="L62" t="n">
+      <c r="I62" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3812,13 +3812,13 @@
         </is>
       </c>
       <c r="D63" s="1" t="n">
-        <v>7.2</v>
+        <v>0.12</v>
       </c>
       <c r="E63" s="1" t="n">
-        <v>6000</v>
+        <v>16100</v>
       </c>
       <c r="F63" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
@@ -3828,16 +3828,16 @@
       <c r="H63" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I63" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" t="n">
-        <v>0</v>
-      </c>
-      <c r="L63" t="n">
+      <c r="I63" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3856,10 +3856,10 @@
         </is>
       </c>
       <c r="D64" s="1" t="n">
-        <v>0.1</v>
+        <v>12.1</v>
       </c>
       <c r="E64" s="1" t="n">
-        <v>17000</v>
+        <v>21100</v>
       </c>
       <c r="F64" s="1" t="n">
         <v>2</v>
@@ -3872,16 +3872,16 @@
       <c r="H64" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I64" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" t="n">
-        <v>0</v>
-      </c>
-      <c r="K64" t="n">
-        <v>0</v>
-      </c>
-      <c r="L64" t="n">
+      <c r="I64" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3900,13 +3900,13 @@
         </is>
       </c>
       <c r="D65" s="1" t="n">
-        <v>6.1</v>
+        <v>5.48</v>
       </c>
       <c r="E65" s="1" t="n">
-        <v>17000</v>
+        <v>11080</v>
       </c>
       <c r="F65" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
@@ -3916,16 +3916,16 @@
       <c r="H65" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I65" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" t="n">
-        <v>0</v>
-      </c>
-      <c r="L65" t="n">
+      <c r="I65" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3944,10 +3944,10 @@
         </is>
       </c>
       <c r="D66" s="1" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="E66" s="1" t="n">
-        <v>17000</v>
+        <v>16200</v>
       </c>
       <c r="F66" s="1" t="n">
         <v>2</v>
@@ -3960,16 +3960,16 @@
       <c r="H66" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I66" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" t="n">
-        <v>0</v>
-      </c>
-      <c r="K66" t="n">
-        <v>0</v>
-      </c>
-      <c r="L66" t="n">
+      <c r="I66" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3988,13 +3988,13 @@
         </is>
       </c>
       <c r="D67" s="1" t="n">
-        <v>7.3</v>
+        <v>11.9</v>
       </c>
       <c r="E67" s="1" t="n">
-        <v>7500</v>
+        <v>21200</v>
       </c>
       <c r="F67" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
@@ -4004,16 +4004,16 @@
       <c r="H67" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K67" t="n">
-        <v>0</v>
-      </c>
-      <c r="L67" t="n">
+      <c r="I67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4032,13 +4032,13 @@
         </is>
       </c>
       <c r="D68" s="1" t="n">
-        <v>8.9</v>
+        <v>5.6</v>
       </c>
       <c r="E68" s="1" t="n">
-        <v>9000</v>
+        <v>11060</v>
       </c>
       <c r="F68" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
@@ -4048,16 +4048,16 @@
       <c r="H68" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I68" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" t="n">
-        <v>0</v>
-      </c>
-      <c r="K68" t="n">
-        <v>0</v>
-      </c>
-      <c r="L68" t="n">
+      <c r="I68" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4076,10 +4076,10 @@
         </is>
       </c>
       <c r="D69" s="1" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="E69" s="1" t="n">
-        <v>18000</v>
+        <v>16300</v>
       </c>
       <c r="F69" s="1" t="n">
         <v>2</v>
@@ -4092,16 +4092,16 @@
       <c r="H69" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I69" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" t="n">
-        <v>0</v>
-      </c>
-      <c r="L69" t="n">
+      <c r="I69" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4120,13 +4120,13 @@
         </is>
       </c>
       <c r="D70" s="1" t="n">
-        <v>7.3</v>
+        <v>12.05</v>
       </c>
       <c r="E70" s="1" t="n">
-        <v>7600</v>
+        <v>21300</v>
       </c>
       <c r="F70" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
@@ -4136,16 +4136,16 @@
       <c r="H70" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I70" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" t="n">
-        <v>0</v>
-      </c>
-      <c r="L70" t="n">
+      <c r="I70" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4164,13 +4164,13 @@
         </is>
       </c>
       <c r="D71" s="1" t="n">
-        <v>9.800000000000001</v>
+        <v>5.52</v>
       </c>
       <c r="E71" s="1" t="n">
-        <v>9000</v>
+        <v>11040</v>
       </c>
       <c r="F71" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
@@ -4180,16 +4180,16 @@
       <c r="H71" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I71" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" t="n">
-        <v>0</v>
-      </c>
-      <c r="L71" t="n">
+      <c r="I71" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
         <v>11</v>
       </c>
       <c r="E72" s="1" t="n">
-        <v>440000</v>
+        <v>315000</v>
       </c>
       <c r="F72" s="1" t="n">
         <v>2</v>
@@ -4224,16 +4224,16 @@
       <c r="H72" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I72" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" t="n">
-        <v>0</v>
-      </c>
-      <c r="K72" t="n">
-        <v>0</v>
-      </c>
-      <c r="L72" t="n">
+      <c r="I72" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4268,16 +4268,16 @@
       <c r="H73" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I73" t="n">
+      <c r="I73" s="1" t="n">
         <v>300000</v>
       </c>
-      <c r="J73" t="n">
-        <v>1</v>
-      </c>
-      <c r="K73" t="n">
-        <v>0</v>
-      </c>
-      <c r="L73" t="n">
+      <c r="J73" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K73" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4299,7 +4299,7 @@
         <v>6.6</v>
       </c>
       <c r="E74" s="1" t="n">
-        <v>1250000</v>
+        <v>895000</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>2</v>
@@ -4312,16 +4312,16 @@
       <c r="H74" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I74" t="n">
-        <v>0</v>
-      </c>
-      <c r="J74" t="n">
-        <v>0</v>
-      </c>
-      <c r="K74" t="n">
-        <v>0</v>
-      </c>
-      <c r="L74" t="n">
+      <c r="I74" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4356,16 +4356,16 @@
       <c r="H75" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I75" t="n">
+      <c r="I75" s="1" t="n">
         <v>770000</v>
       </c>
-      <c r="J75" t="n">
-        <v>1</v>
-      </c>
-      <c r="K75" t="n">
-        <v>0</v>
-      </c>
-      <c r="L75" t="n">
+      <c r="J75" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K75" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="1" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>